<commit_message>
chore: cập nhật BCTC đầy đủ 2026-09-23
</commit_message>
<xml_diff>
--- a/financials/FPT/FPT.xlsx
+++ b/financials/FPT/FPT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="4695" windowWidth="15120" windowHeight="8205" tabRatio="600" firstSheet="4" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="balance_sheet" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,10 +13,6 @@
     <sheet name="Dự báo tăng trưởng" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Hiệu quả thực hiện kế hoạch" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId7"/>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +29,7 @@
   </numFmts>
   <fonts count="18">
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -117,14 +113,14 @@
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <b val="1"/>
       <color theme="1"/>
@@ -253,7 +249,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -315,6 +311,9 @@
     <xf numFmtId="165" fontId="15" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="41" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="41" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -535,95 +534,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
-    <sheetNames>
-      <sheetName val="Sheet1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="2">
-          <cell r="D2">
-            <v>66400</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
-    <sheetNames>
-      <sheetName val="CĐKT"/>
-      <sheetName val="KQHĐKD"/>
-      <sheetName val="LCTT"/>
-      <sheetName val="Tổng quan"/>
-      <sheetName val="Dự báo tăng trưởng"/>
-      <sheetName val="Cơ cấu DT, LN"/>
-      <sheetName val="Hiệu quả thực hiện KH của DN"/>
-      <sheetName val="Phân tích"/>
-      <sheetName val="Chỉ số"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="4">
-          <cell r="E4">
-            <v>29830</v>
-          </cell>
-          <cell r="F4">
-            <v>35657</v>
-          </cell>
-          <cell r="G4">
-            <v>44010</v>
-          </cell>
-          <cell r="H4">
-            <v>52618</v>
-          </cell>
-          <cell r="I4">
-            <v>62849</v>
-          </cell>
-          <cell r="J4">
-            <v>70113</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="E18">
-            <v>5263</v>
-          </cell>
-          <cell r="F18">
-            <v>6337</v>
-          </cell>
-          <cell r="G18">
-            <v>7662</v>
-          </cell>
-          <cell r="H18">
-            <v>9203</v>
-          </cell>
-          <cell r="I18">
-            <v>11070</v>
-          </cell>
-          <cell r="J18">
-            <v>13044</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6920,11 +6830,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J83"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="38.33203125" customWidth="1" min="1" max="1"/>
+    <col width="38.375" customWidth="1" min="1" max="1"/>
     <col width="19" bestFit="1" customWidth="1" min="2" max="9"/>
-    <col width="20.5546875" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="20.5" bestFit="1" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -8294,7 +8204,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="1" s="34">
+    <row r="39" ht="15" customFormat="1" customHeight="1" s="34">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Vốn chủ sở hữu</t>
@@ -8334,7 +8244,7 @@
       </c>
       <c r="J39" s="44" t="n"/>
     </row>
-    <row r="40" customFormat="1" s="34">
+    <row r="40" ht="15" customFormat="1" customHeight="1" s="34">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Lợi ích cổ đông không kiểm soát</t>
@@ -8388,7 +8298,7 @@
       <c r="H41" s="9" t="n"/>
       <c r="I41" s="9" t="n"/>
     </row>
-    <row r="42" customFormat="1" s="34">
+    <row r="42" ht="15" customFormat="1" customHeight="1" s="34">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Doanh thu thuần</t>
@@ -8469,7 +8379,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" customFormat="1" s="34">
+    <row r="44" ht="15" customFormat="1" customHeight="1" s="34">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Lợi nhuận gộp</t>
@@ -8664,7 +8574,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" customFormat="1" s="34">
+    <row r="49" ht="15" customFormat="1" customHeight="1" s="34">
       <c r="A49" s="35" t="inlineStr">
         <is>
           <t>Lãi/(lỗ) trước thuế</t>
@@ -8706,7 +8616,7 @@
         <v>11629000000000</v>
       </c>
     </row>
-    <row r="50" customFormat="1" s="34">
+    <row r="50" ht="15" customFormat="1" customHeight="1" s="34">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Lãi/(lỗ) thuần sau thuế</t>
@@ -8745,7 +8655,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" customFormat="1" s="34">
+    <row r="51" ht="15" customFormat="1" customHeight="1" s="34">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>Lợi nhuận của Cổ đông của Công ty mẹ</t>
@@ -9929,7 +9839,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="12.75"/>
   <cols>
     <col width="14" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
     <col width="19" bestFit="1" customWidth="1" style="31" min="2" max="5"/>
@@ -9984,21 +9894,17 @@
           <t>Thị giá</t>
         </is>
       </c>
-      <c r="B3" s="26">
-        <f>[1]Sheet1!$D$2</f>
-        <v/>
-      </c>
-      <c r="C3" s="26">
-        <f>[1]Sheet1!$D$2</f>
-        <v/>
-      </c>
-      <c r="D3" s="26">
-        <f>[1]Sheet1!$D$2</f>
-        <v/>
-      </c>
-      <c r="E3" s="26">
-        <f>[1]Sheet1!$D$2</f>
-        <v/>
+      <c r="B3" s="26" t="n">
+        <v>66400</v>
+      </c>
+      <c r="C3" s="26" t="n">
+        <v>66400</v>
+      </c>
+      <c r="D3" s="26" t="n">
+        <v>66400</v>
+      </c>
+      <c r="E3" s="26" t="n">
+        <v>66400</v>
       </c>
     </row>
     <row r="4">
@@ -10030,17 +9936,17 @@
           <t>VCSH</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="47" t="n">
         <v>40122000000000</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="47" t="n">
         <v>40996000000000</v>
       </c>
-      <c r="D6" s="27">
+      <c r="D6" s="47">
         <f>$C$6*(($E$6/$C$6)^(1/2))</f>
         <v/>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="47" t="n">
         <v>46100000000000</v>
       </c>
     </row>
@@ -10050,17 +9956,17 @@
           <t>LICĐKKS</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="47" t="n">
         <v>1170000000000</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="47" t="n">
         <v>1144000000000</v>
       </c>
-      <c r="D7" s="27">
+      <c r="D7" s="47">
         <f>D6*0.03</f>
         <v/>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="47">
         <f>E6*0.03</f>
         <v/>
       </c>
@@ -10071,19 +9977,19 @@
           <t>BV</t>
         </is>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="47">
         <f>B6-B7</f>
         <v/>
       </c>
-      <c r="C8" s="27">
+      <c r="C8" s="47">
         <f>C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="27">
+      <c r="D8" s="47">
         <f>D6-D7</f>
         <v/>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="47">
         <f>E6-E7</f>
         <v/>
       </c>
@@ -10094,19 +10000,19 @@
           <t>BVPS</t>
         </is>
       </c>
-      <c r="B9" s="29">
+      <c r="B9" s="48">
         <f>B8/B2</f>
         <v/>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="48">
         <f>C8/C2</f>
         <v/>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="48">
         <f>D8/D2</f>
         <v/>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="48">
         <f>E8/E2</f>
         <v/>
       </c>
@@ -10141,15 +10047,15 @@
         </is>
       </c>
       <c r="B12" s="25" t="n"/>
-      <c r="C12" s="27">
+      <c r="C12" s="47">
         <f>(2568+2487+2503+2435)*1000000000</f>
         <v/>
       </c>
-      <c r="D12" s="27">
+      <c r="D12" s="47">
         <f>$C$12*(($E$12/$C$12)^(1/2))</f>
         <v/>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="47">
         <f>chi_so_tai_chinh!J51</f>
         <v/>
       </c>
@@ -10160,18 +10066,18 @@
           <t>EPS</t>
         </is>
       </c>
-      <c r="B13" s="29" t="n">
+      <c r="B13" s="48" t="n">
         <v>5687</v>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="48">
         <f>C12/C2</f>
         <v/>
       </c>
-      <c r="D13" s="29">
+      <c r="D13" s="48">
         <f>$C$13*(($E$13/$C$13)^(1/2))</f>
         <v/>
       </c>
-      <c r="E13" s="29">
+      <c r="E13" s="48">
         <f>E12/E2</f>
         <v/>
       </c>
@@ -10212,11 +10118,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="12.75"/>
   <cols>
-    <col width="29.33203125" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
-    <col width="8.109375" bestFit="1" customWidth="1" style="31" min="2" max="8"/>
-    <col width="8.88671875" customWidth="1" style="31" min="9" max="16384"/>
+    <col width="29.375" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
+    <col width="8.125" bestFit="1" customWidth="1" style="31" min="2" max="8"/>
+    <col width="8.875" customWidth="1" style="31" min="9" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10249,25 +10155,25 @@
           <t>Doanh thu kế hoạch</t>
         </is>
       </c>
-      <c r="B2" s="37" t="n">
+      <c r="B2" s="49" t="n">
         <v>32450</v>
       </c>
-      <c r="C2" s="37" t="n">
+      <c r="C2" s="49" t="n">
         <v>34720</v>
       </c>
-      <c r="D2" s="37" t="n">
+      <c r="D2" s="49" t="n">
         <v>42420</v>
       </c>
-      <c r="E2" s="37" t="n">
+      <c r="E2" s="49" t="n">
         <v>52289</v>
       </c>
-      <c r="F2" s="37" t="n">
+      <c r="F2" s="49" t="n">
         <v>61850</v>
       </c>
-      <c r="G2" s="37" t="n">
+      <c r="G2" s="49" t="n">
         <v>75400</v>
       </c>
-      <c r="H2" s="37" t="n">
+      <c r="H2" s="49" t="n">
         <v>58580</v>
       </c>
     </row>
@@ -10277,31 +10183,31 @@
           <t>Doanh thu thuần</t>
         </is>
       </c>
-      <c r="B3" s="37">
-        <f>([2]KQHĐKD!E4*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="C3" s="37">
-        <f>([2]KQHĐKD!F4*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="D3" s="37">
-        <f>([2]KQHĐKD!G4*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="E3" s="37">
-        <f>([2]KQHĐKD!H4*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="F3" s="37">
-        <f>([2]KQHĐKD!I4*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="G3" s="37">
-        <f>([2]KQHĐKD!J4*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="H3" s="37">
+      <c r="B3" s="49">
+        <f>chi_so_tai_chinh!D42/1000000000</f>
+        <v/>
+      </c>
+      <c r="C3" s="49">
+        <f>chi_so_tai_chinh!E42/1000000000</f>
+        <v/>
+      </c>
+      <c r="D3" s="49">
+        <f>chi_so_tai_chinh!F42/1000000000</f>
+        <v/>
+      </c>
+      <c r="E3" s="49">
+        <f>chi_so_tai_chinh!G42/1000000000</f>
+        <v/>
+      </c>
+      <c r="F3" s="49">
+        <f>chi_so_tai_chinh!H42/1000000000</f>
+        <v/>
+      </c>
+      <c r="G3" s="49">
+        <f>chi_so_tai_chinh!I42/1000000000</f>
+        <v/>
+      </c>
+      <c r="H3" s="49">
         <f>12486+13810</f>
         <v/>
       </c>
@@ -10347,25 +10253,25 @@
           <t>Lợi nhuận trước thuế kế hoạch</t>
         </is>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="49" t="n">
         <v>5510</v>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="C5" s="49" t="n">
         <v>6210</v>
       </c>
-      <c r="D5" s="37" t="n">
+      <c r="D5" s="49" t="n">
         <v>7618</v>
       </c>
-      <c r="E5" s="37" t="n">
+      <c r="E5" s="49" t="n">
         <v>9055</v>
       </c>
-      <c r="F5" s="37" t="n">
+      <c r="F5" s="49" t="n">
         <v>10875</v>
       </c>
-      <c r="G5" s="37" t="n">
+      <c r="G5" s="49" t="n">
         <v>13395</v>
       </c>
-      <c r="H5" s="37" t="n">
+      <c r="H5" s="49" t="n">
         <v>11629</v>
       </c>
     </row>
@@ -10375,31 +10281,31 @@
           <t>Tổng lợi nhuận kế toán trước thuế</t>
         </is>
       </c>
-      <c r="B6" s="37">
-        <f>([2]KQHĐKD!E18*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="C6" s="37">
-        <f>([2]KQHĐKD!F18*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="D6" s="37">
-        <f>([2]KQHĐKD!G18*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="E6" s="37">
-        <f>([2]KQHĐKD!H18*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="F6" s="37">
-        <f>([2]KQHĐKD!I18*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="G6" s="37">
-        <f>([2]KQHĐKD!J18*1000)/1000</f>
-        <v/>
-      </c>
-      <c r="H6" s="37">
+      <c r="B6" s="49">
+        <f>chi_so_tai_chinh!D49/1000000000</f>
+        <v/>
+      </c>
+      <c r="C6" s="49">
+        <f>chi_so_tai_chinh!E49/1000000000</f>
+        <v/>
+      </c>
+      <c r="D6" s="49">
+        <f>chi_so_tai_chinh!F49/1000000000</f>
+        <v/>
+      </c>
+      <c r="E6" s="49">
+        <f>chi_so_tai_chinh!G49/1000000000</f>
+        <v/>
+      </c>
+      <c r="F6" s="49">
+        <f>chi_so_tai_chinh!H49/1000000000</f>
+        <v/>
+      </c>
+      <c r="G6" s="49">
+        <f>chi_so_tai_chinh!I49/1000000000</f>
+        <v/>
+      </c>
+      <c r="H6" s="49">
         <f>2804+2910</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
chore: cập nhật BCTC đầy đủ 2026-10-29
</commit_message>
<xml_diff>
--- a/financials/FPT/FPT.xlsx
+++ b/financials/FPT/FPT.xlsx
@@ -836,16 +836,16 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0</v>
+        <v>5568623727137</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0</v>
+        <v>6708978162325</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0</v>
+        <v>12435918124269</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0</v>
+        <v>20730720735456</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>0</v>
@@ -866,10 +866,18 @@
           <t>Đầu tư ngắn hạn</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F7" s="4" t="n">
         <v>0</v>
       </c>
@@ -1231,16 +1239,16 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>0</v>
+        <v>1144102797190</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0</v>
+        <v>996357466471</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0</v>
+        <v>588320170446</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0</v>
+        <v>580281075542</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>0</v>
@@ -1354,10 +1362,18 @@
           <t>Tài sản lưu động khác</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
+      <c r="B23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F23" s="4" t="n">
         <v>0</v>
       </c>
@@ -2246,16 +2262,16 @@
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>335327364</v>
+        <v>37229856110</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>0</v>
+        <v>40251284363</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>258372310</v>
+        <v>139469584405</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>87366215294</v>
+        <v>182211531443</v>
       </c>
       <c r="F52" s="4" t="n">
         <v>149305200735</v>
@@ -2896,10 +2912,18 @@
           <t>Thuế thu nhập hoãn lại</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr"/>
-      <c r="C73" s="4" t="inlineStr"/>
-      <c r="D73" s="4" t="inlineStr"/>
-      <c r="E73" s="4" t="inlineStr"/>
+      <c r="B73" s="4" t="n">
+        <v>335327364</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>258372310</v>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>87366215294</v>
+      </c>
       <c r="F73" s="4" t="n">
         <v>149305200735</v>
       </c>
@@ -3633,16 +3657,16 @@
         </is>
       </c>
       <c r="B97" s="4" t="n">
-        <v>0</v>
+        <v>5568623727137</v>
       </c>
       <c r="C97" s="4" t="n">
-        <v>0</v>
+        <v>6708978162325</v>
       </c>
       <c r="D97" s="4" t="n">
-        <v>200000000</v>
+        <v>12435918124269</v>
       </c>
       <c r="E97" s="4" t="n">
-        <v>200000000</v>
+        <v>20730720735456</v>
       </c>
       <c r="F97" s="4" t="n">
         <v>10200000000</v>
@@ -3911,10 +3935,18 @@
           <t>Đầu tư nắm giữ đến ngày đáo hạn</t>
         </is>
       </c>
-      <c r="B106" s="4" t="inlineStr"/>
-      <c r="C106" s="4" t="inlineStr"/>
-      <c r="D106" s="4" t="inlineStr"/>
-      <c r="E106" s="4" t="inlineStr"/>
+      <c r="B106" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" s="4" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>200000000</v>
+      </c>
       <c r="F106" s="4" t="n">
         <v>10200000000</v>
       </c>
@@ -4182,10 +4214,18 @@
           <t>Cổ phiếu ưu đãi</t>
         </is>
       </c>
-      <c r="B115" s="4" t="inlineStr"/>
-      <c r="C115" s="4" t="inlineStr"/>
-      <c r="D115" s="4" t="inlineStr"/>
-      <c r="E115" s="4" t="inlineStr"/>
+      <c r="B115" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C115" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F115" s="4" t="n">
         <v>0</v>
       </c>

</xml_diff>